<commit_message>
Add new account sampling population
</commit_message>
<xml_diff>
--- a/Ale-InspectionSuccursales.xlsx
+++ b/Ale-InspectionSuccursales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://peakgroup0-my.sharepoint.com/personal/aduplaga_peakgroup_com/Documents/source/repos/Compliance_BRN_Samples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="8_{C08D7061-467F-49D9-BA49-F53AFEEB14EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E513BA19-0B24-44AF-B81C-0775CF184015}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="8_{C08D7061-467F-49D9-BA49-F53AFEEB14EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DD8A2B7-38B4-4EAD-82B6-0193990170E2}"/>
   <bookViews>
     <workbookView xWindow="15195" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{CD0190AD-07ED-4561-9762-79CFF99B3F22}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="58">
   <si>
     <t>Analyse d'affaire - échantillonnage pour inspection des succursales SPP</t>
   </si>
@@ -320,6 +320,9 @@
   </si>
   <si>
     <t>35,40,45,50,100</t>
+  </si>
+  <si>
+    <t>Done</t>
   </si>
 </sst>
 </file>
@@ -789,24 +792,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70FE22A9-16AA-4CFE-9D55-23CD5B07B211}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="16.2" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.09765625" customWidth="1"/>
     <col min="2" max="2" width="42.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="54" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="54" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -814,15 +817,18 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="129.6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="129.6" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="129.6" x14ac:dyDescent="0.35">
+      <c r="C7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="129.6" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>4</v>
       </c>
@@ -830,28 +836,37 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="108" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="108" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>6</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="108" x14ac:dyDescent="0.35">
+      <c r="C11" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="108" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" ht="108" x14ac:dyDescent="0.35">
+      <c r="C13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="108" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>25</v>
+      </c>
+      <c r="C15" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="72" x14ac:dyDescent="0.35">
@@ -1262,14 +1277,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0ef1a97a-1525-4ed2-8a8e-361511404792">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="c0fd1c75-a352-4d68-8516-d309e31bea90" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1502,21 +1515,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0ef1a97a-1525-4ed2-8a8e-361511404792">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="c0fd1c75-a352-4d68-8516-d309e31bea90" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62DBD3C3-9991-4938-9B89-33B1DA4B502F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A1D9A5-C798-4B8F-8C4B-30C2548BF16C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0ef1a97a-1525-4ed2-8a8e-361511404792"/>
-    <ds:schemaRef ds:uri="c0fd1c75-a352-4d68-8516-d309e31bea90"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1541,9 +1553,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A1D9A5-C798-4B8F-8C4B-30C2548BF16C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62DBD3C3-9991-4938-9B89-33B1DA4B502F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0ef1a97a-1525-4ed2-8a8e-361511404792"/>
+    <ds:schemaRef ds:uri="c0fd1c75-a352-4d68-8516-d309e31bea90"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>